<commit_message>
Dados reais, comparacao entre ferramentas e correcoes encontradas nos testes
- amostra de 100 avaliacoes do B2W-Reviews01 (CC BY-NC-SA 4.0) e planilha de rotulagem
- respostas de ChatGPT, Claude e Gemini web nas mesmas 20 avaliacoes e modo
  concordancia no comparar_ferramentas.py
- agente avaliado nas 8 perguntas com dados reais; resultados em resultados/
- correcoes: datas ISO lidas como dia/mes; busca quebrando no limite de embeddings;
  classificacao insistindo apos o fim da cota (agora para, guarda e retoma com --continuar);
  modelos lite sem a opcao de desligar raciocinio
- modelo reserva passa a ser o gemini-3.5-flash-lite
</commit_message>
<xml_diff>
--- a/data/rotulagem/planilha_rotulagem.xlsx
+++ b/data/rotulagem/planilha_rotulagem.xlsx
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M44"/>
+  <dimension ref="A1:M101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="2" max="2"/>
@@ -806,7 +806,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Veio faltando o refrigerante e ninguém respondeu no chat.</t>
+          <t>Entrega rápida, produto compatível com o preço,mas uma panela veio riscada dentro, deixando a peça com aparência ruim.</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Tudo certo com o pedido, chegou no horário.</t>
+          <t>Meu produto veio com a cor diferente. Comprei sabendo que seria aquele rosa claro que tá mostrando e veio rosa Pink. Também veio faltando a bolsa. Quando vcs vão me enviar a bolsa?</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Achei caro, mas a qualidade compensa.</t>
+          <t>Horrível não recomendo americanas a ninguém,pois não me retornaram o e-mail e nada. Fiz o pagamento quando chegou na minha casa o produto estava gasto,riscado,sujo,com cola  Simplesmente não era igual o anuncio,parecia até que estava usado que simplesmente colocaram na caixa e me entregaram</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Comida maravilhosa mas demorou 40 min pra sair.</t>
+          <t>O depilador é ótimo, ergonômico, leve e não dói. Funcionou muito bem para mim. Super recomendo pela relação custo benefício!</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Que maravilha, cheguei e a mesa estava grudenta e cheia de moscas.</t>
+          <t>Alongador atendeu perfeitamente. Proporcionou maior conforto</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Preço muito alto pelo tamanho do lanche, não compensa.</t>
+          <t>Gostei bastante, chegou bem antes do previsto!o preço estava ótimo,alisa bem os cabelos, minha filha adorou,gosto muito de comprar nas Americanas!</t>
         </is>
       </c>
     </row>
@@ -866,7 +866,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Salão limpinho e música ambiente agradável.</t>
+          <t>Adorei...muito bem acabado e bonito...entrega bem rápida...</t>
         </is>
       </c>
     </row>
@@ -876,7 +876,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Embalagem vazou e sujou toda a sacola.</t>
+          <t>Produto bom e barato. Proporciona uma boa impressão - não idêntica à original -  a um custo baixo.</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Fui no sábado à noite com minha família.</t>
+          <t>Não posso avaliar, porque infelizmente a entrega de vocês é péssima, e ainda não recebi o produto. Pior! Não recebo satisfação, do que esta acontecendo. Me sentido lesado...</t>
         </is>
       </c>
     </row>
@@ -896,7 +896,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Cardápio variado e porções bem servidas pelo preço.</t>
+          <t>Muito bom recomendo a todos, fácil instalação e água realmente gelada.</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Melhor pizza da cidade, sem dúvidas!!!</t>
+          <t>muito bom de comunicação, chega antes do prazo e em perfeitas condições.</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Lugar limpo e organizado, atendimento nota 10.</t>
+          <t>Produto e entrega no prazo espero q continue assim</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Ambiente bonito, mas a fila no caixa é enorme nos fins de semana.</t>
+          <t>péssimo produto, os botões ficar falhando e o frete é caro, não gaste seu dinheiro com essa porcaria!!</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Os donos são muito simpáticos e o pão de queijo é o melhor!</t>
+          <t>Maravilhosa desliza super bem , é bivolt esquenta super rápido quem comprar não vai se arrepender</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Promoção de terça vale muito a pena, preço ótimo.</t>
+          <t>Fiz a compra há quase 2 meses e ainda não foi entregue. Espero que não venha com nenhum problema pra valer a pena.</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Me ligue no [TELEFONE] para conversar sobre parceria.</t>
+          <t>Comprei a philco 20 polegada o controle vem c smart mas nao funciona o smart o q faço?qr aproveitar o YouTube.</t>
         </is>
       </c>
     </row>
@@ -966,7 +966,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Atendimento rápido, comida boa, mas o lugar é muito barulhento.</t>
+          <t>Muito bom, 100% satisfeito, só esperava um pouco mais da bateria...</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Esperei 30 minutos na mesa e ninguém veio atender.</t>
+          <t>Ótimo celular, os pontos negativos são que a câmera as vezes borra a foto e o celular esquenta quando utilizados vários aplicativos.</t>
         </is>
       </c>
     </row>
@@ -986,7 +986,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Parabéns, esperei só 50 minutos por um x-salada. Show de bola 👏</t>
+          <t>excelente leitura -  recomendo com certeza  Philips Yancey é um dos melhores autores  cristãos da atualidade</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Batata frita sem sal e o molho acabou.</t>
+          <t>O produto é excelente e a entrega foi bem antes do previsto, adorei.</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>O suco veio aguado e a coxinha fria.</t>
+          <t>Produto muito bom igual a descrição o tecido é bom a cor é igual</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Gostei, mas achei a porção pequena.</t>
+          <t>ELE NÃO GELA A ÁGUA. SÓ SAI ÁGUA NATURAL. GOSTARIA DE SABER SE POSSO TROCAR. O QUE FAÇO. QUERIA SABER POR QUE ESTÁ ESCRITO QUE SAI ÁGUA GELADA MAS NÃO SAI?</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Cobraram a taxa de serviço sem avisar, achei desonesto.</t>
+          <t>Caneca bonita e veio muito bem embalada. Só a qualidade da estampa que não me agradou muito</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Entrega super rápida e embalagem caprichada, parabéns à equipe!</t>
+          <t>Gostaria de opinar sobre o produto, porém a primeira entrega veio com o produto errado, solicitei a troca e estou ainda aguardando. o interessante é que comprei a mais de um mês (14/12) e nada ainda.  A crítica não é ao produto, mais para aqueles que venderam...</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>top demais, atendimento brabo e lanche monstro</t>
+          <t>Exatamente igual a foto!!! Ficou lindo na minha sala. A entrega mto antes do prazo!!!!</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Ótimo atendimento, só que não. Fui ignorado no balcão.</t>
+          <t>O aparelho é ótimo, câmera excelente tem muitas funções não deixa nada a desejar, entrega dentro do prazo , parabéns a equipe,lojas Americanas.</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Pedi sem cebola e veio com cebola. De novo.</t>
+          <t>Porém a entrega demora muito quando comparado a outros sites.</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Estacionamento difícil e o ar-condicionado não funcionava.</t>
+          <t>Tamanho ideal para família pequena. Bonita e ótimo custo benefício.</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Hambúrguer muito saboroso e chegou quentinho, recomendo!</t>
+          <t>O livro é uma obra repleta de referências aos anos 80 e ao mesmo tempo uma história jovial com momentos leves e tensões que vão fazer seus olhos não descansarem. Uma das minhas melhores leituras. Recomendo.  A entrega da Americanas.com também está de parabéns. Além da rapidez, o produto chegou muito bem embalado.</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>O entregador foi educado, mas o lanche veio amassado.</t>
+          <t>Jogo muito bom,já to zerando pela segunda vez e não travou nem se quer uma vez. Excelente</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Demora absurda no delivery, 1h20 de espera, e o motoboy ainda reclamou da gorjeta.</t>
+          <t>Deveria ter mais cola pq usei poucas vezes e já nao cola mais</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1116,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>zuado demais, pedido trocado e frio</t>
+          <t>Após pesquisar muito sobre o aparelho decidi comprar e estou muito satisfeita! Imagem e som ótimos. Entrega dentro do prazo.</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>O garçom [NOME] super atencioso, ambiente agradável.</t>
+          <t>vcs poderia dar mais cupus de descontos pra quem compra mais ou vale compra pra ser aceito em qlq produto  eu mesmo compro muito de voces  grato romualdo</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>A comida estava ok, o atendimento que deixou a desejar.</t>
+          <t>bom dia! o headset esta com  mal contato, não consigo entrar em contato com vcs!!</t>
         </is>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>A atendente foi grossa quando perguntei sobre o cardápio.</t>
+          <t>O PRODUTO É DIFERENTE DO ORIGINAL. O cone de engate e maior, tive que usar uma arroela para dar aperto.</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1156,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Banheiro sujo e sem papel. Comida ok.</t>
+          <t>Um bom celular com boa duração da bateria, fotos boas lindo design e conectá rápido ao WiFi</t>
         </is>
       </c>
     </row>
@@ -1166,7 +1166,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Nunca mais peço aí. Carne crua no hambúrguer.</t>
+          <t>Em resumo, não cumpre o que promete. Já pedi orientações para devolvê-lo. No aguardo.</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Bom.</t>
+          <t>Maravilhoso, recomendo sim o produto, chegou na minha casa antes do prazo estabelecido, muito bom mesmo!</t>
         </is>
       </c>
     </row>
@@ -1186,7 +1186,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Preço subiu muito de um mês pro outro, o lanche continua o mesmo.</t>
+          <t>É muito bom comprar na americanas, pois tudo vem certinho e tudo em perfeito estado.  E este produto em específico, foi entregue aqui na minha mão aqui em casa. Muito bom isso.</t>
         </is>
       </c>
     </row>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Lanche bom, preço razoável. Nada de especial.</t>
+          <t>Neste último produto,  a qualidade ficou à desejar.</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1206,7 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Pastel crocante e recheado, voltarei com certeza.</t>
+          <t>Comprei este kit acreditando na marca pois ela e fabricada pela Boch, so que os acessessorios são de pessima qualidade, as brocas que acompanhavam meu kit ou quebram ou entortam, as pontas da parafusadeira simplismente espanam o parafuso e quebram. Resumindo uma porcaria, não recomendo a ninguem.</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>mó brisa esse açaí, preço justo, recomendo dms</t>
+          <t>O produto veio com a caixa violada, sem o lacre da embalagem. eu não recomendo a compra pelas americanas, fora a demora na entrega o produto chegou com a violada.</t>
         </is>
       </c>
     </row>
@@ -1226,40 +1226,610 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Demorou mais de uma hora pra chegar e a batata veio murcha.</t>
+          <t>Livro mt bom, para estudantes e profissionais da fono. Com ilustrações, livro bem objetivo. Gostei bastante</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Produto de qualidade. Chegou super rápido. Tenho um Samsung S7, e comprei esse pois o outro descarrega muito rápido e esquenta as vezes. Para o dia a dia, essa é a melhor opção. A bateria dura o dia todo, usando quase todas as redes sociais. Amei meu J5 pro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Eu odiei meu Produto, pois veio totalmente diferente do que eu pedir, como o tecido, o mode e ate a cor, não foi a que esta mostrando na imagem do produto original. Portanto estou bem decepcionado com a loja e o site em que fiz minha primeira compra, por essa razão, não compro e nem recomendo a loja e o site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>O celular chegou muito rápido, tem ótimo desempenho e custo-benefício.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Tudo certo conforme o anúncio. O produto chegou rápido e em perfeitas condições.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Produto com preço bem barato, só espero não ter problemas com instalação</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>nao recebi produto...trocaram telefone sem mesmo notificar as  lojas AAMERICANAS essa loja nao ê recomendável Magazine Romero ...nao comprem paguei por um produto e trocaram</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Ótimas fotos, muito rápido, bom espaço, boa bateria  só vem muitos aplicativos instalados, mas dá para desativar no gerenciador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Lindo,muito grande,achei que era menor.Da pra usar até como cachecol.Tecido de qualidade.Recomendo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Comprei essa tv depois de pesquisar muito qual seria a melhor opção para acompanhar minhas series do Netflix, certamente essa é a que tem o melhor custo beneficio! O fator de vir com dois controles também é muito interessante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Gostei bastante do produto. Já recomendo às minhas amigas</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>não gostei material da impressora muito frágil. cartuchos preto e colorido vieram vazios. não tive como testar por falta da tinta. não recomendo</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Produto entregue no prazo.  E muito bom. ..........................</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Produto realmente original, com data de fabricação muito proxima da data de venda, encaixa perfeitamente e dura como durava a bateria original. Recomendo o vendedor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Espanta morcegos... Mais precisa ficar ligado por uns 2 meses. Caso contrário eles voltam. Não faz barulho aos ouvidos humanos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Jogo bom para quem gosta de ação e aventura,............................................................................................................................................................</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Vi algumas avaliações sobre o produto reclamando de lentidão, de falta de gravador de dvd, etc. Para a finalidade que eu comprei o notebook, ele me satisfaz plenamente. Não vou usar jogos nele, nem vou usar programas de design pesados.   Para o que quero: navegar na internet, fazer compras, administrar minhas contas bancárias, ele é bem rápido e seguro. Gostei muito.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Produto ótimo,   de acordo com o solicitado e em perfeitas condições. Entregue antes do prazo previsto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Recebi o produto muito,muito antes da data prevista para entrega. Recomendo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>QUERO ELOGIAR A ENTREGA QUE FOI MUITO RÁPIDA. EXCELENTE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>O preço do produto e equiparado a sua qualidade. O copo e mais frágil do que os outros modelos. Mas pelo preço que se paga e só ter cuidado que vc terá seu produto por bastante tempo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Tive problemas no produto. Canto da mesa veio avariado e o pé da mesa veio com um modelo totalmente diferente ( veio na cor branco). Caso consiga resolver junto a empresa modifico minha opinião.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Amei o perfume! É marcante, fixação muito boa e dura muito na pele. Produto original!</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Mta demora na entrega nem recebi mais já me arrependi de ter comprado! Nunca esperei tanto uma entrega pela americnas.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Custo benefício, dentro do valor pago é satisfatório o que proporciona</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>O Smartphone Xiaomi Redmi me surpreendeu muito, melhor do que muitos se não todos os celulares na sua faixa de preço, muito bom</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>A impressora Epson Ecotank L120 Colorida é excelente produto eu recomendo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Excelente produto!! Adorei a escova alisadora mondial!!!</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>livro muito bom, explica  como interagir com os bebês numa fase fundamental da vida, principalmente quando os bebês ficam longe dos pais, quando estes estão no trabalho..</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>O produto deve ser bom, "deve ser" pois ainda nao recebi. A entrega esta atrasada. Nunca mais compro em lojas que utilizem a Directlog para entrega.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>Muito bom atendeu a todas as minhas nescessidades ,indico a todos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Produto branco na parte interior,  isso não foi mencionado na descrição. Possui tonalidades diferentes de uma parte para outra. Alguns quebradinhos do transportes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>Imagem perfeita. Funções de smart excepcional . superou as expectativas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>Produto muito bom pelo valor! Entrega: muito agiu foi muito bom comprar com a Americanas. Recomendo para todos!</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>Ótimo produto, fácil de configurar entradas hdmi e usb bem localizadas, recomendo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>Excelente produto! Adorando o meu ,muito eficiente !</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>bateria dura bem para 3.000 mAh, celular é rápido, a câmera é boa e tem um ótimo preço. Excelente trabalho da Direct, empresa que faz a entrega. Não paguei o frete, ou seja econômica com previsão de entrega para 10 a 13 dias e o produto chegou em 7 dias úteis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>O produto até o momento atende bem pra quem usa todo dia, porém se for encher a mochila seu tempo de uso vai diminuir. O material da mochila é bom, a alça não é muito confortável mas é resistente. Se o objetivo é usar levando notebook aconselho outro produto, o compartimento de notebook é bem ruim, a espuma é muito fina e não protege bem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>Super recomendo! Celular excelente!!!   Muito bom !!!!!!!!!!!!</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>O produto não gela a água, apenas resfria, demora muito para resfriar novamente, após o uso. Não tem controle de temperatura.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>Ótimo exatamente o que eu queria optei em retirada  Loja Americanas ,chegou muito antes do previsto eu Super Recomendo este liquidificador sem contar que ele é LINDO... MUITO BOM E BATE AS FRUTAS SEM DEIXAR PEDACINHOS ....MARAVILHOS PODEM APOSTAR !</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Produto muito bom Entrega rápida  Entrega no prazo determinado Recomendo a todos</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>Comprei 2 controles. Um deles está com problemas. Não faz a conexão com o portão de forma alguma.  O outro está tudo OK! Nem sei como resolver.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>Ótima qualidade, ótimo material, lindo .. Só veio com o pistão quebrado, não tá segurando a porta basculante ;( Mas de resto muito bom</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>Muito bom o celular. O único ponto negativo é o grande tempo que leva para recarregar a bateria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Chegou antes do prazo estimado,, esse eu recomendo. Vendedor atencioso e competente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>Muito pratico e facil de usar bom para todos os dias</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>comprei no sábado e recebi na quinta, produto integro! fogão menor do que os de mesa em inox. possui chamas bem altas e forte! ainda não testei o forno , mas parece ser bom. o fogão possui um visual lindo!!! super fácil de limpar, só não sei o forno. pelo designer e poder das chamas o preço compensa. ideal para lugares e família pequena. amei...</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>O produto é bom, recomendo, bom de tamanho, não toma muito espaço.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>A balança oscila muito os valores, tem uma variação de até 1 kg. Para que quer acompanhar o peso não compensa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Atendeu bem as minhas expectativas, custo benefício ótimo!! compro de novo se precisar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>Pensei que o produto fosse original e não é, péssimo material já sou a tampa do fone em 1 semana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>Muito bom o aparelho e boa potencia, recomendo o aparelho.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>Fiquei impressionado com o ruído baixo e a potencia. Além de ser linda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>Ar condicionado silencioso, resfria bem, atendeu as minhas expectativas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>Maravilhoso, veste muito bem. Uso 48 ficou perfeito.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>Fiz o pedido dia (23-04-2018), antes de confirmar a compra, estava explicito no site, que vocês iriam entregar de 7 á 10 dias úteis, e bem, hoje já é dia (27-04-2018), já se passou exata uma semana do lançamento e até hoje, ainda está na nota fiscal emitida, detalhe: desde segunda-feira passada, dia ( 23-04-2018). Depois da efetuação do pedido, a data foi postergada para dia (30-04-2018), passados 3-4 dias, a Americanas me adia novamente a data de entrega, para até agora, dia (02-04-2018).  Comprei na pré-venda, com a certeza de pegar o jogo o quanto antes possível, bem perto de seu lançamento, mas até hoje estou esperando e quero saber Americanas, quanto tempo a mais terei que esperar?  Se vocês oferecem para seus clientes o serviço de pré-venda e não cumprem com a palavra, vocês não estão respeitando as pessoas que são fundamentais para a sustentação e para o crescimento da Americanas, que são seus clientes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>O produto é de fato o que eu esperava que ele fosse,cumpre tudo o que está descrito em sua "ficha técnica" e atende todas as minhas expectativas...</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="10">
-    <dataValidation sqref="C2:C44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C2:C101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"positivo,neutro,negativo"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"x"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"x"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"x"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"x"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"x"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"x"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"x"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
-    <dataValidation sqref="L2:L44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"sim,não"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>